<commit_message>
feat: expeditor loading 5.2.0 nakladnoy, refusals, warehouse template fixes
- Add ex-5.2.0 expeditor loading template, fill, merge rebuild (Excel repair fix)

- Warehouse nakladnoy assets, zip patch, repair/sanitize, bulk export UI

- Client refusals module (API, migration, frontend), seed and audit scripts

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/backend/assets/nakladnoy/warehouse/600-wh-6.0.xlsx
+++ b/backend/assets/nakladnoy/warehouse/600-wh-6.0.xlsx
@@ -2298,13 +2298,9 @@
   <mergeCells>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:C2"/>
     <mergeCell ref="A3:B3"/>
-    <mergeCell ref="C3:C3"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:C4"/>
     <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:C5"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="D1:D6"/>
     <mergeCell ref="E1:E6"/>
@@ -2380,7 +2376,6 @@
     <mergeCell ref="B69:C69"/>
     <mergeCell ref="B70:C70"/>
     <mergeCell ref="B71:C71"/>
-    <mergeCell ref="B72:B72"/>
   </mergeCells>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.2" right="0.2" top="0.2" bottom="0.2" header="0.3" footer="0.3"/>

</xml_diff>